<commit_message>
beta vs ke graph added
</commit_message>
<xml_diff>
--- a/output/capm_master_dataset.xlsx
+++ b/output/capm_master_dataset.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CAPM_Master" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="CAPM_Master" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -490,7 +490,7 @@
         <v>0.194022</v>
       </c>
       <c r="H2" t="n">
-        <v>1.356916</v>
+        <v>1.356915</v>
       </c>
       <c r="I2" t="n">
         <v>0.346221</v>
@@ -523,7 +523,7 @@
         <v>0.194022</v>
       </c>
       <c r="H3" t="n">
-        <v>0.5695249999999999</v>
+        <v>0.569524</v>
       </c>
       <c r="I3" t="n">
         <v>0.19345</v>
@@ -589,7 +589,7 @@
         <v>-0.014424</v>
       </c>
       <c r="H5" t="n">
-        <v>0.9803500000000001</v>
+        <v>0.980349</v>
       </c>
       <c r="I5" t="n">
         <v>0.06783500000000001</v>
@@ -610,7 +610,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.529852</v>
+        <v>0.529853</v>
       </c>
       <c r="E6" t="n">
         <v>0.067552</v>
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.048701</v>
+        <v>0.0487</v>
       </c>
       <c r="E8" t="n">
         <v>0.31388</v>
@@ -688,7 +688,7 @@
         <v>0.228329</v>
       </c>
       <c r="H8" t="n">
-        <v>0.16881</v>
+        <v>0.168809</v>
       </c>
       <c r="I8" t="n">
         <v>0.124095</v>
@@ -721,7 +721,7 @@
         <v>0.228329</v>
       </c>
       <c r="H9" t="n">
-        <v>0.5797870000000001</v>
+        <v>0.579788</v>
       </c>
       <c r="I9" t="n">
         <v>0.217933</v>
@@ -787,7 +787,7 @@
         <v>-0.11811</v>
       </c>
       <c r="H11" t="n">
-        <v>0.182055</v>
+        <v>0.182054</v>
       </c>
       <c r="I11" t="n">
         <v>0.055999</v>
@@ -820,7 +820,7 @@
         <v>-0.11811</v>
       </c>
       <c r="H12" t="n">
-        <v>0.559611</v>
+        <v>0.559612</v>
       </c>
       <c r="I12" t="n">
         <v>0.011406</v>
@@ -853,7 +853,7 @@
         <v>-0.11811</v>
       </c>
       <c r="H13" t="n">
-        <v>0.882927</v>
+        <v>0.882926</v>
       </c>
       <c r="I13" t="n">
         <v>-0.026781</v>
@@ -907,7 +907,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>-0.065197</v>
+        <v>-0.065196</v>
       </c>
       <c r="E15" t="n">
         <v>0.030133</v>
@@ -952,7 +952,7 @@
         <v>-0.041605</v>
       </c>
       <c r="H16" t="n">
-        <v>1.029246</v>
+        <v>1.029245</v>
       </c>
       <c r="I16" t="n">
         <v>0.028917</v>
@@ -1018,7 +1018,7 @@
         <v>0.218987</v>
       </c>
       <c r="H18" t="n">
-        <v>0.300731</v>
+        <v>0.300733</v>
       </c>
       <c r="I18" t="n">
         <v>0.133329</v>
@@ -1051,10 +1051,10 @@
         <v>0.218987</v>
       </c>
       <c r="H19" t="n">
-        <v>0.754908</v>
+        <v>0.754907</v>
       </c>
       <c r="I19" t="n">
-        <v>0.232788</v>
+        <v>0.232787</v>
       </c>
     </row>
     <row r="20">
@@ -1150,7 +1150,7 @@
         <v>-0.045677</v>
       </c>
       <c r="H22" t="n">
-        <v>1.045938</v>
+        <v>1.045937</v>
       </c>
       <c r="I22" t="n">
         <v>0.029414</v>
@@ -1216,7 +1216,7 @@
         <v>0.051035</v>
       </c>
       <c r="H24" t="n">
-        <v>0.428511</v>
+        <v>0.428512</v>
       </c>
       <c r="I24" t="n">
         <v>0.091054</v>
@@ -1249,10 +1249,10 @@
         <v>0.051035</v>
       </c>
       <c r="H25" t="n">
-        <v>1.350934</v>
+        <v>1.350933</v>
       </c>
       <c r="I25" t="n">
-        <v>0.138131</v>
+        <v>0.13813</v>
       </c>
     </row>
     <row r="26">
@@ -1303,7 +1303,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0.759651</v>
+        <v>0.75965</v>
       </c>
       <c r="E27" t="n">
         <v>0.149016</v>
@@ -1369,7 +1369,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>1.19751</v>
+        <v>1.197509</v>
       </c>
       <c r="E29" t="n">
         <v>0.241193</v>
@@ -1381,7 +1381,7 @@
         <v>0.179303</v>
       </c>
       <c r="H29" t="n">
-        <v>0.980949</v>
+        <v>0.98095</v>
       </c>
       <c r="I29" t="n">
         <v>0.237777</v>
@@ -1414,7 +1414,7 @@
         <v>0.179303</v>
       </c>
       <c r="H30" t="n">
-        <v>0.564079</v>
+        <v>0.564078</v>
       </c>
       <c r="I30" t="n">
         <v>0.163031</v>
@@ -1447,7 +1447,7 @@
         <v>0.179303</v>
       </c>
       <c r="H31" t="n">
-        <v>1.486641</v>
+        <v>1.48664</v>
       </c>
       <c r="I31" t="n">
         <v>0.328449</v>
@@ -1480,7 +1480,7 @@
         <v>-0.028593</v>
       </c>
       <c r="H32" t="n">
-        <v>1.109417</v>
+        <v>1.109418</v>
       </c>
       <c r="I32" t="n">
         <v>0.040161</v>
@@ -1567,7 +1567,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>0.642611</v>
+        <v>0.64261</v>
       </c>
       <c r="E35" t="n">
         <v>0.200278</v>
@@ -1579,7 +1579,7 @@
         <v>0.128042</v>
       </c>
       <c r="H35" t="n">
-        <v>0.9531230000000001</v>
+        <v>0.953124</v>
       </c>
       <c r="I35" t="n">
         <v>0.194276</v>
@@ -1612,7 +1612,7 @@
         <v>0.128042</v>
       </c>
       <c r="H36" t="n">
-        <v>0.647058</v>
+        <v>0.647057</v>
       </c>
       <c r="I36" t="n">
         <v>0.155087</v>
@@ -1633,7 +1633,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>1.907296</v>
+        <v>1.907295</v>
       </c>
       <c r="E37" t="n">
         <v>0.200278</v>
@@ -1666,7 +1666,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>0.559864</v>
+        <v>0.559863</v>
       </c>
       <c r="E38" t="n">
         <v>0.088048</v>
@@ -1678,7 +1678,7 @@
         <v>0.018588</v>
       </c>
       <c r="H38" t="n">
-        <v>0.952142</v>
+        <v>0.952143</v>
       </c>
       <c r="I38" t="n">
         <v>0.087158</v>
@@ -1711,7 +1711,7 @@
         <v>0.018588</v>
       </c>
       <c r="H39" t="n">
-        <v>0.7867960000000001</v>
+        <v>0.786795</v>
       </c>
       <c r="I39" t="n">
         <v>0.08408499999999999</v>
@@ -1777,7 +1777,7 @@
         <v>0.040057</v>
       </c>
       <c r="H41" t="n">
-        <v>1.101489</v>
+        <v>1.10149</v>
       </c>
       <c r="I41" t="n">
         <v>0.109154</v>
@@ -1810,7 +1810,7 @@
         <v>0.040057</v>
       </c>
       <c r="H42" t="n">
-        <v>0.803161</v>
+        <v>0.80316</v>
       </c>
       <c r="I42" t="n">
         <v>0.097204</v>

</xml_diff>

<commit_message>
beta vs ke added
</commit_message>
<xml_diff>
--- a/output/capm_master_dataset.xlsx
+++ b/output/capm_master_dataset.xlsx
@@ -490,7 +490,7 @@
         <v>0.194022</v>
       </c>
       <c r="H2" t="n">
-        <v>1.356915</v>
+        <v>1.356916</v>
       </c>
       <c r="I2" t="n">
         <v>0.346221</v>
@@ -559,7 +559,7 @@
         <v>1.066275</v>
       </c>
       <c r="I4" t="n">
-        <v>0.28983</v>
+        <v>0.289831</v>
       </c>
     </row>
     <row r="5">
@@ -577,7 +577,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.536284</v>
+        <v>0.536283</v>
       </c>
       <c r="E5" t="n">
         <v>0.067552</v>
@@ -589,7 +589,7 @@
         <v>-0.014424</v>
       </c>
       <c r="H5" t="n">
-        <v>0.980349</v>
+        <v>0.9803500000000001</v>
       </c>
       <c r="I5" t="n">
         <v>0.06783500000000001</v>
@@ -610,7 +610,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.529853</v>
+        <v>0.529852</v>
       </c>
       <c r="E6" t="n">
         <v>0.067552</v>
@@ -622,7 +622,7 @@
         <v>-0.014424</v>
       </c>
       <c r="H6" t="n">
-        <v>0.541374</v>
+        <v>0.541373</v>
       </c>
       <c r="I6" t="n">
         <v>0.074167</v>
@@ -643,7 +643,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.309658</v>
+        <v>0.309657</v>
       </c>
       <c r="E7" t="n">
         <v>0.067552</v>
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.0487</v>
+        <v>0.048701</v>
       </c>
       <c r="E8" t="n">
         <v>0.31388</v>
@@ -688,7 +688,7 @@
         <v>0.228329</v>
       </c>
       <c r="H8" t="n">
-        <v>0.168809</v>
+        <v>0.16881</v>
       </c>
       <c r="I8" t="n">
         <v>0.124095</v>
@@ -721,7 +721,7 @@
         <v>0.228329</v>
       </c>
       <c r="H9" t="n">
-        <v>0.579788</v>
+        <v>0.5797870000000001</v>
       </c>
       <c r="I9" t="n">
         <v>0.217933</v>
@@ -787,7 +787,7 @@
         <v>-0.11811</v>
       </c>
       <c r="H11" t="n">
-        <v>0.182054</v>
+        <v>0.182055</v>
       </c>
       <c r="I11" t="n">
         <v>0.055999</v>
@@ -820,7 +820,7 @@
         <v>-0.11811</v>
       </c>
       <c r="H12" t="n">
-        <v>0.559612</v>
+        <v>0.559611</v>
       </c>
       <c r="I12" t="n">
         <v>0.011406</v>
@@ -853,7 +853,7 @@
         <v>-0.11811</v>
       </c>
       <c r="H13" t="n">
-        <v>0.882926</v>
+        <v>0.882927</v>
       </c>
       <c r="I13" t="n">
         <v>-0.026781</v>
@@ -886,7 +886,7 @@
         <v>-0.041605</v>
       </c>
       <c r="H14" t="n">
-        <v>0.237681</v>
+        <v>0.237682</v>
       </c>
       <c r="I14" t="n">
         <v>0.06185</v>
@@ -907,7 +907,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>-0.065196</v>
+        <v>-0.065197</v>
       </c>
       <c r="E15" t="n">
         <v>0.030133</v>
@@ -973,7 +973,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.557725</v>
+        <v>0.5577260000000001</v>
       </c>
       <c r="E17" t="n">
         <v>0.28646</v>
@@ -1051,10 +1051,10 @@
         <v>0.218987</v>
       </c>
       <c r="H19" t="n">
-        <v>0.754907</v>
+        <v>0.754908</v>
       </c>
       <c r="I19" t="n">
-        <v>0.232787</v>
+        <v>0.232788</v>
       </c>
     </row>
     <row r="20">
@@ -1150,7 +1150,7 @@
         <v>-0.045677</v>
       </c>
       <c r="H22" t="n">
-        <v>1.045937</v>
+        <v>1.045938</v>
       </c>
       <c r="I22" t="n">
         <v>0.029414</v>
@@ -1183,7 +1183,7 @@
         <v>0.051035</v>
       </c>
       <c r="H23" t="n">
-        <v>1.165591</v>
+        <v>1.165592</v>
       </c>
       <c r="I23" t="n">
         <v>0.128671</v>
@@ -1249,10 +1249,10 @@
         <v>0.051035</v>
       </c>
       <c r="H25" t="n">
-        <v>1.350933</v>
+        <v>1.350934</v>
       </c>
       <c r="I25" t="n">
-        <v>0.13813</v>
+        <v>0.138131</v>
       </c>
     </row>
     <row r="26">
@@ -1348,10 +1348,10 @@
         <v>0.088404</v>
       </c>
       <c r="H28" t="n">
-        <v>1.424935</v>
+        <v>1.424936</v>
       </c>
       <c r="I28" t="n">
-        <v>0.186582</v>
+        <v>0.186583</v>
       </c>
     </row>
     <row r="29">
@@ -1414,7 +1414,7 @@
         <v>0.179303</v>
       </c>
       <c r="H30" t="n">
-        <v>0.564078</v>
+        <v>0.564079</v>
       </c>
       <c r="I30" t="n">
         <v>0.163031</v>
@@ -1447,7 +1447,7 @@
         <v>0.179303</v>
       </c>
       <c r="H31" t="n">
-        <v>1.48664</v>
+        <v>1.486641</v>
       </c>
       <c r="I31" t="n">
         <v>0.328449</v>
@@ -1513,7 +1513,7 @@
         <v>-0.028593</v>
       </c>
       <c r="H33" t="n">
-        <v>0.657155</v>
+        <v>0.657156</v>
       </c>
       <c r="I33" t="n">
         <v>0.053093</v>
@@ -1612,7 +1612,7 @@
         <v>0.128042</v>
       </c>
       <c r="H36" t="n">
-        <v>0.647057</v>
+        <v>0.647058</v>
       </c>
       <c r="I36" t="n">
         <v>0.155087</v>
@@ -1633,7 +1633,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>1.907295</v>
+        <v>1.907296</v>
       </c>
       <c r="E37" t="n">
         <v>0.200278</v>
@@ -1666,7 +1666,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>0.559863</v>
+        <v>0.559864</v>
       </c>
       <c r="E38" t="n">
         <v>0.088048</v>
@@ -1711,7 +1711,7 @@
         <v>0.018588</v>
       </c>
       <c r="H39" t="n">
-        <v>0.786795</v>
+        <v>0.7867960000000001</v>
       </c>
       <c r="I39" t="n">
         <v>0.08408499999999999</v>
@@ -1777,7 +1777,7 @@
         <v>0.040057</v>
       </c>
       <c r="H41" t="n">
-        <v>1.10149</v>
+        <v>1.101489</v>
       </c>
       <c r="I41" t="n">
         <v>0.109154</v>

</xml_diff>